<commit_message>
Remove company-specific public assumptions and clarify personal authorship
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R09eb9cc9cfc94f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R48b29b4980e5441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rd9d5021ae4db4233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant" sheetId="4" r:id="R07bf7b1e0f5443a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R64c3a1efa1df4566"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R3f30f29e7c654881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R2771b231b9574791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rfec8358089b948e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="Rb7289f092d934d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Reaa0020b0c6241df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant" sheetId="4" r:id="Rb750ccf55f95421a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R0a4f181c0e0344d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R2a147ef9eba14e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R11bdd89afaeb45f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -524,7 +524,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="275">
+  <x:cellXfs count="278">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1113,6 +1113,11 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1361,17 +1366,17 @@
       <x:c r="G2" s="100"/>
       <x:c r="H2" s="43"/>
     </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="101" t="str">
-        <x:v>Portfolio demonstration only - generalized architecture, synthetic values, no production connection</x:v>
-      </x:c>
-      <x:c r="B3" s="101"/>
-      <x:c r="C3" s="101"/>
-      <x:c r="D3" s="101"/>
-      <x:c r="E3" s="101"/>
-      <x:c r="F3" s="101"/>
-      <x:c r="G3" s="101"/>
-      <x:c r="H3" s="44"/>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" s="80" t="str">
+        <x:v>Personal portfolio case study by Thomas Ryan. Not an official PepperBall publication. Synthetic demonstration; no production connection.</x:v>
+      </x:c>
+      <x:c r="B3" s="80"/>
+      <x:c r="C3" s="80"/>
+      <x:c r="D3" s="80"/>
+      <x:c r="E3" s="80"/>
+      <x:c r="F3" s="80"/>
+      <x:c r="G3" s="80"/>
+      <x:c r="H3" s="277"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="45"/>
@@ -2002,7 +2007,7 @@
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="121" t="str">
-        <x:v>30 hours/week of reporting effort addressed (20 supervisor + 10 manager), representing about $52K in modeled annual labor value under documented assumptions.</x:v>
+        <x:v>30 hours/week of reporting effort addressed, representing about $52K in modeled annual labor-capacity value. Underlying company-specific assumptions are omitted from this public case study.</x:v>
       </x:c>
       <x:c r="B14" s="121"/>
       <x:c r="C14" s="121"/>
@@ -2699,7 +2704,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="146" t="str">
-        <x:v>Impact model - editable assumptions</x:v>
+        <x:v>Impact overview - qualified public estimates</x:v>
       </x:c>
       <x:c r="B1" s="146"/>
       <x:c r="C1" s="146"/>
@@ -2720,26 +2725,26 @@
       <x:c r="H2" s="146"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
-      <x:c r="A3" s="148" t="str">
-        <x:v>Planning scenarios only. Inputs are editable; outputs are formulas, not booked results.</x:v>
-      </x:c>
-      <x:c r="B3" s="148"/>
-      <x:c r="C3" s="148"/>
-      <x:c r="D3" s="148"/>
-      <x:c r="E3" s="148"/>
-      <x:c r="F3" s="148"/>
-      <x:c r="G3" s="148"/>
-      <x:c r="H3" s="148"/>
+      <x:c r="A3" s="89" t="str">
+        <x:v>Underlying company-specific assumptions are omitted from this public case study.</x:v>
+      </x:c>
+      <x:c r="B3" s="89"/>
+      <x:c r="C3" s="89"/>
+      <x:c r="D3" s="89"/>
+      <x:c r="E3" s="89"/>
+      <x:c r="F3" s="89"/>
+      <x:c r="G3" s="89"/>
+      <x:c r="H3" s="89"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="150" t="str">
-        <x:v>MODEL</x:v>
+        <x:v>VALUE AREA</x:v>
       </x:c>
       <x:c r="B5" s="150" t="str">
-        <x:v>INPUT</x:v>
+        <x:v>MEASURE</x:v>
       </x:c>
       <x:c r="C5" s="150" t="str">
-        <x:v>VALUE</x:v>
+        <x:v>ESTIMATE</x:v>
       </x:c>
       <x:c r="D5" s="150" t="str">
         <x:v>UNIT</x:v>
@@ -2748,7 +2753,7 @@
         <x:v>OUTPUT</x:v>
       </x:c>
       <x:c r="G5" s="156" t="str">
-        <x:v>FORMULA</x:v>
+        <x:v>BASIS / LIMIT</x:v>
       </x:c>
       <x:c r="H5" s="156" t="str">
         <x:v>RESULT</x:v>
@@ -2756,112 +2761,108 @@
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="160" t="str">
-        <x:v>Labor</x:v>
+        <x:v>Core reporting</x:v>
       </x:c>
       <x:c r="B6" s="160" t="str">
-        <x:v>Supervisor hours/week</x:v>
-      </x:c>
-      <x:c r="C6" s="161" t="n">
-        <x:v>20</x:v>
+        <x:v>Weekly capacity</x:v>
+      </x:c>
+      <x:c r="C6" s="275" t="n">
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D6" s="160" t="str">
-        <x:v>hours</x:v>
+        <x:v>hours/week</x:v>
       </x:c>
       <x:c r="F6" s="163" t="str">
         <x:v>Labor hours/year</x:v>
       </x:c>
       <x:c r="G6" s="169" t="str">
-        <x:v>(20 + 10) hours × 52 weeks</x:v>
+        <x:v>Modeled annual capacity</x:v>
       </x:c>
       <x:c r="H6" s="164" t="n">
-        <x:f>(C6+C7)*C8</x:f>
         <x:v>1560</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="160" t="str">
-        <x:v>Labor</x:v>
+        <x:v>Core reporting</x:v>
       </x:c>
       <x:c r="B7" s="160" t="str">
-        <x:v>Manager hours/week</x:v>
-      </x:c>
-      <x:c r="C7" s="161" t="n">
-        <x:v>10</x:v>
+        <x:v>Annual capacity</x:v>
+      </x:c>
+      <x:c r="C7" s="275" t="n">
+        <x:v>1560</x:v>
       </x:c>
       <x:c r="D7" s="160" t="str">
-        <x:v>hours</x:v>
+        <x:v>hours/year</x:v>
       </x:c>
       <x:c r="F7" s="163" t="str">
         <x:v>Modeled labor value</x:v>
       </x:c>
       <x:c r="G7" s="169" t="str">
-        <x:v>Labor hours × $33.33/hour</x:v>
+        <x:v>Approximate modeled value</x:v>
       </x:c>
       <x:c r="H7" s="165" t="n">
-        <x:f>H6*C9</x:f>
-        <x:v>51994.799999999996</x:v>
+        <x:v>52000</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="160" t="str">
-        <x:v>Labor</x:v>
+        <x:v>Core reporting</x:v>
       </x:c>
       <x:c r="B8" s="160" t="str">
-        <x:v>Weeks/year</x:v>
-      </x:c>
-      <x:c r="C8" s="161" t="n">
-        <x:v>52</x:v>
+        <x:v>Modeled annual value</x:v>
+      </x:c>
+      <x:c r="C8" s="275" t="n">
+        <x:v>52000</x:v>
       </x:c>
       <x:c r="D8" s="160" t="str">
-        <x:v>weeks</x:v>
+        <x:v>USD/year (approx.)</x:v>
       </x:c>
       <x:c r="F8" s="163" t="str">
         <x:v>Estimated assistant retrieval reduction</x:v>
       </x:c>
       <x:c r="G8" s="169" t="str">
-        <x:v>(25 minutes - 2 minutes) ÷ 25 minutes</x:v>
+        <x:v>Representative comparison; not a controlled benchmark</x:v>
       </x:c>
       <x:c r="H8" s="166" t="n">
-        <x:f>(C10-C11)/C10</x:f>
-        <x:v>0.92</x:v>
+        <x:v>0.9</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="160" t="str">
-        <x:v>Labor</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B9" s="160" t="str">
-        <x:v>Blended hourly value</x:v>
-      </x:c>
-      <x:c r="C9" s="161" t="n">
-        <x:v>33.33</x:v>
+        <x:v>Annual upper bound</x:v>
+      </x:c>
+      <x:c r="C9" s="275" t="n">
+        <x:v>227500</x:v>
       </x:c>
       <x:c r="D9" s="160" t="str">
-        <x:v>$/hour</x:v>
+        <x:v>production units/year</x:v>
       </x:c>
       <x:c r="F9" s="163" t="str">
         <x:v>Machine-visibility production-unit opportunity</x:v>
       </x:c>
       <x:c r="G9" s="169" t="str">
-        <x:v>5 minutes ÷ 60 × 1,000 production units × 52.5 × 52</x:v>
+        <x:v>Upper bound, not recovered production</x:v>
       </x:c>
       <x:c r="H9" s="164" t="n">
-        <x:f>C12/60*C13*C14*C15</x:f>
         <x:v>227500</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="160" t="str">
-        <x:v>Reporting Assistant</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B10" s="160" t="str">
-        <x:v>Baseline search</x:v>
-      </x:c>
-      <x:c r="C10" s="161" t="n">
-        <x:v>25</x:v>
+        <x:v>Modeled margin</x:v>
+      </x:c>
+      <x:c r="C10" s="275" t="n">
+        <x:v>205000</x:v>
       </x:c>
       <x:c r="D10" s="160" t="str">
-        <x:v>minutes</x:v>
+        <x:v>USD/year (approx.)</x:v>
       </x:c>
       <x:c r="F10"/>
       <x:c r="G10" s="170"/>
@@ -2871,105 +2872,64 @@
         <x:v>Reporting Assistant</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>Bounded retrieval</x:v>
-      </x:c>
-      <x:c r="C11" s="161" t="n">
-        <x:v>2</x:v>
+        <x:v>Retrieval improvement</x:v>
+      </x:c>
+      <x:c r="C11" s="276" t="n">
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="D11" s="160" t="str">
-        <x:v>minutes</x:v>
+        <x:v>estimated reduction</x:v>
       </x:c>
       <x:c r="F11" s="157" t="str">
         <x:v>Machine-visibility contribution-margin opportunity</x:v>
       </x:c>
       <x:c r="G11" s="99" t="str">
-        <x:v>Production-unit opportunity × $0.90/unit</x:v>
+        <x:v>Approximate upper bound, not realized margin</x:v>
       </x:c>
       <x:c r="H11" s="167" t="n">
-        <x:f>H9*C16</x:f>
-        <x:v>204750</x:v>
+        <x:v>205000</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="160" t="str">
-        <x:v>Machine visibility</x:v>
-      </x:c>
-      <x:c r="B12" s="160" t="str">
-        <x:v>Response improvement</x:v>
-      </x:c>
-      <x:c r="C12" s="161" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D12" s="160" t="str">
-        <x:v>minutes</x:v>
-      </x:c>
+      <x:c r="A12" s="160"/>
+      <x:c r="B12" s="160"/>
+      <x:c r="C12" s="161"/>
+      <x:c r="D12" s="160"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="160" t="str">
-        <x:v>Machine visibility</x:v>
-      </x:c>
-      <x:c r="B13" s="160" t="str">
-        <x:v>Throughput</x:v>
-      </x:c>
-      <x:c r="C13" s="161" t="n">
-        <x:v>1000</x:v>
-      </x:c>
-      <x:c r="D13" s="160" t="str">
-        <x:v>production units/hour/machine</x:v>
-      </x:c>
+      <x:c r="A13" s="160"/>
+      <x:c r="B13" s="160"/>
+      <x:c r="C13" s="161"/>
+      <x:c r="D13" s="160"/>
       <x:c r="F13" s="168" t="str">
-        <x:v>Limitations: representative time study, role-rate assumptions, event frequency, throughput, response improvement, and margin are scenario inputs. The labor-capacity and machine-visibility value pools are separate and are not added together. Outputs are not realized savings, guaranteed production, or autonomous outcomes.</x:v>
+        <x:v>Underlying company-specific assumptions are omitted from this public case study. The labor-capacity and machine-visibility models are separate and are not added together. Estimates do not establish company approval.</x:v>
       </x:c>
       <x:c r="G13" s="168"/>
       <x:c r="H13" s="168"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="160" t="str">
-        <x:v>Machine visibility</x:v>
-      </x:c>
-      <x:c r="B14" s="160" t="str">
-        <x:v>Events/week</x:v>
-      </x:c>
-      <x:c r="C14" s="161" t="n">
-        <x:v>52.5</x:v>
-      </x:c>
-      <x:c r="D14" s="160" t="str">
-        <x:v>events</x:v>
-      </x:c>
+      <x:c r="A14" s="160"/>
+      <x:c r="B14" s="160"/>
+      <x:c r="C14" s="161"/>
+      <x:c r="D14" s="160"/>
       <x:c r="F14" s="168"/>
       <x:c r="G14" s="168"/>
       <x:c r="H14" s="168"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="160" t="str">
-        <x:v>Machine visibility</x:v>
-      </x:c>
-      <x:c r="B15" s="160" t="str">
-        <x:v>Weeks/year</x:v>
-      </x:c>
-      <x:c r="C15" s="161" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="D15" s="160" t="str">
-        <x:v>weeks</x:v>
-      </x:c>
+      <x:c r="A15" s="160"/>
+      <x:c r="B15" s="160"/>
+      <x:c r="C15" s="161"/>
+      <x:c r="D15" s="160"/>
       <x:c r="F15" s="168"/>
       <x:c r="G15" s="168"/>
       <x:c r="H15" s="168"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="160" t="str">
-        <x:v>Machine visibility</x:v>
-      </x:c>
-      <x:c r="B16" s="160" t="str">
-        <x:v>Contribution margin</x:v>
-      </x:c>
-      <x:c r="C16" s="161" t="n">
-        <x:v>0.9</x:v>
-      </x:c>
-      <x:c r="D16" s="160" t="str">
-        <x:v>$/unit</x:v>
-      </x:c>
+      <x:c r="A16" s="160"/>
+      <x:c r="B16" s="160"/>
+      <x:c r="C16" s="161"/>
+      <x:c r="D16" s="160"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="245" t="str">
@@ -3025,7 +2985,7 @@
       </x:c>
       <x:c r="E20" s="271" t="n">
         <x:f>'Impact Model'!H7</x:f>
-        <x:v>51994.799999999996</x:v>
+        <x:v>52000</x:v>
       </x:c>
       <x:c r="F20" s="261" t="str">
         <x:v>Modeled labor-capacity value</x:v>
@@ -3053,7 +3013,7 @@
       </x:c>
       <x:c r="E21" s="272" t="n">
         <x:f>'Impact Model'!H11</x:f>
-        <x:v>204750</x:v>
+        <x:v>205000</x:v>
       </x:c>
       <x:c r="F21" s="264" t="str">
         <x:v>Modeled upper bound</x:v>
@@ -3074,7 +3034,7 @@
       </x:c>
       <x:c r="C22" s="273" t="n">
         <x:f>'Impact Model'!H8</x:f>
-        <x:v>0.92</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="D22" s="267" t="str">
         <x:v>retrieval reduction</x:v>

</xml_diff>